<commit_message>
update to Labs 3 and HW 4 and Lab5-1
</commit_message>
<xml_diff>
--- a/book/modules/data/Cedar_average_monthly_waterbalance.xlsx
+++ b/book/modules/data/Cedar_average_monthly_waterbalance.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jdlund/Documents/CEE348_EnvE_Environmental_flows_class/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jdlund/Documents/CEE348_EnvE_Environmental_flows_class/Homework/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BAA98B4-F983-5147-9B62-E2F4DE957B78}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{806F34BD-23FB-894F-85A6-E66B1DA179D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4880" yWindow="1000" windowWidth="27640" windowHeight="15780" xr2:uid="{74B3E998-A0A8-3C43-89F0-0B04BD3A310A}"/>
+    <workbookView xWindow="2340" yWindow="1800" windowWidth="27640" windowHeight="15780" xr2:uid="{74B3E998-A0A8-3C43-89F0-0B04BD3A310A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -95,15 +95,6 @@
     <t>Average Streamflow (cfs)</t>
   </si>
   <si>
-    <t xml:space="preserve">Note: Streamflow is from USGS gage: 12116400 </t>
-  </si>
-  <si>
-    <t>for years 2001 to 2019</t>
-  </si>
-  <si>
-    <t>The gage is listed as having area of 217 km^2</t>
-  </si>
-  <si>
     <t xml:space="preserve">Note: Monthly ET is from climatological maps here:  http://www.cpc.ncep.noaa.gov/soilmst/e.shtml </t>
   </si>
   <si>
@@ -132,6 +123,15 @@
   </si>
   <si>
     <t>in mm/year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note: Streamflow is from USGS gage: 12116500 </t>
+  </si>
+  <si>
+    <t>The gage is listed as having area of 218 km^2</t>
+  </si>
+  <si>
+    <t>for water yrs 2001 to 2023</t>
   </si>
 </sst>
 </file>
@@ -188,9 +188,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -228,7 +228,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -334,7 +334,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -476,7 +476,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -488,30 +488,31 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="32.33203125" customWidth="1"/>
+    <col min="4" max="4" width="14.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -552,7 +553,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -596,7 +597,7 @@
         <v>55.6</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -640,7 +641,7 @@
         <v>39.5</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -684,53 +685,54 @@
         <v>101.13</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>19</v>
       </c>
       <c r="B10">
-        <v>218</v>
+        <v>589</v>
       </c>
       <c r="C10">
-        <v>141</v>
+        <v>471</v>
       </c>
       <c r="D10">
-        <v>132</v>
+        <v>402</v>
       </c>
       <c r="E10">
-        <v>130</v>
+        <v>365</v>
       </c>
       <c r="F10">
-        <v>142</v>
+        <v>390</v>
       </c>
       <c r="G10">
-        <v>105</v>
+        <v>295</v>
       </c>
       <c r="H10">
-        <v>55</v>
+        <v>114</v>
       </c>
       <c r="I10">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="J10">
-        <v>49</v>
+        <v>87</v>
       </c>
       <c r="K10">
-        <v>69</v>
+        <v>233</v>
       </c>
       <c r="L10">
-        <v>196</v>
+        <v>514</v>
       </c>
       <c r="M10">
-        <v>153</v>
-      </c>
-      <c r="N10">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+        <v>457</v>
+      </c>
+      <c r="N10" s="1">
+        <f>AVERAGE(B10:M10)</f>
+        <v>330.58333333333331</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B11">
         <v>3</v>
@@ -772,46 +774,42 @@
         <f>AVERAGE(B11:L11)</f>
         <v>28.09090909090909</v>
       </c>
-      <c r="O11">
-        <f>SUM(B11:M11)</f>
-        <v>311</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13" t="s">
+        <v>31</v>
+      </c>
+      <c r="I13" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>20</v>
       </c>
-      <c r="C13" t="s">
-        <v>21</v>
-      </c>
-      <c r="E13" t="s">
-        <v>22</v>
-      </c>
-      <c r="I13" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="O17" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B18">
         <v>0.61</v>
@@ -859,7 +857,7 @@
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B19">
         <v>0</v>

</xml_diff>